<commit_message>
Add 2025 pace and % comparison columns to Dudu's orthopedics sheet
Same sheet, no new tab: 2025 sales, half-year-equivalent pace, and
2026-vs-pace percentage, alongside the existing orthopedic/sales
ranking and gap columns.
</commit_message>
<xml_diff>
--- a/kirill/outputs/2026-08-01-ביצועי-סניפים-לפי-סוכן.xlsx
+++ b/kirill/outputs/2026-08-01-ביצועי-סניפים-לפי-סוכן.xlsx
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1284" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1287" uniqueCount="463">
   <si>
     <t xml:space="preserve">ביצועי סניפים לפי סוכן — דודו (Top 20 לפי מכירות 2026)</t>
   </si>
@@ -160,7 +160,7 @@
 (מכירות מול אורתופדיה)</t>
   </si>
   <si>
-    <t xml:space="preserve">הערה: הדירוג בעמודה A ובעמודה E הוא דירוג יחסי בין 68 סניפי דודו בלבד (לא הדירוג הכללי ברשת). פער = דירוג מכירות פחות דירוג אורתופדיה; פער חיובי וגדול = הסניף חזק באורתופדיה יחסית לסניפי דודו האחרים אך מוכר פחות טוב יחסית אליהם (פוטנציאל לא ממומש). שורות עם פער &gt;= 10 מודגשות (הסף נבחר לפי התפלגות בפועל: פערים בין -14 ל-16, ממוצע 0, סטיית תקן כ-5).</t>
+    <t xml:space="preserve">הערה: הדירוג בעמודה A ובעמודה H הוא דירוג יחסי בין 68 סניפי דודו בלבד (לא הדירוג הכללי ברשת). פער (עמודה I) = דירוג מכירות פחות דירוג אורתופדיה; פער חיובי וגדול = הסניף חזק באורתופדיה יחסית לסניפי דודו האחרים אך מוכר פחות טוב יחסית אליהם (פוטנציאל לא ממומש). זו מדידה נפרדת לחלוטין מעמודת "2026 מול קצב 2025 (%)" (עמודה G), שמשווה כל סניף לקצב המכירות שלו-עצמו אשתקד, ולא משתתפת בחישוב הפער. שורות עם פער &gt;= 10 מודגשות (הסף נבחר לפי התפלגות בפועל: פערים בין -14 ל-16, ממוצע 0, סטיית תקן כ-5). קצב 2025 = מכירות 2025 (שנה מלאה) חלקי 12 כפול 6, כדי להשוות לחצי-שנה של 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">חנויות</t>
@@ -2741,15 +2741,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2761,6 +2763,9 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -2784,9 +2789,18 @@
         <v>5</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="I4" s="4" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2806,12 +2820,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A5,מקור!$L$2:$L$309,0)),"")</f>
         <v>40303.1</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A5,מקור!$L$2:$L$309,0)),"")</f>
+        <v>70289.5</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <f aca="false">IFERROR(E5/12*6,"")</f>
+        <v>35144.75</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <f aca="false">IFERROR(D5/F5-1,"")</f>
+        <v>0.146774411540842</v>
+      </c>
+      <c r="H5" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A5,מקור!$L$2:$L$309,0)),"")</f>
         <v>1</v>
       </c>
-      <c r="F5" s="9" t="n">
-        <f aca="false">IFERROR(E5-A5,"")</f>
+      <c r="I5" s="9" t="n">
+        <f aca="false">IFERROR(H5-A5,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -2831,12 +2857,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A6,מקור!$L$2:$L$309,0)),"")</f>
         <v>30919.3</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A6,מקור!$L$2:$L$309,0)),"")</f>
+        <v>52742</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <f aca="false">IFERROR(E6/12*6,"")</f>
+        <v>26371</v>
+      </c>
+      <c r="G6" s="7" t="n">
+        <f aca="false">IFERROR(D6/F6-1,"")</f>
+        <v>0.17247355049107</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A6,מקור!$L$2:$L$309,0)),"")</f>
         <v>6</v>
       </c>
-      <c r="F6" s="9" t="n">
-        <f aca="false">IFERROR(E6-A6,"")</f>
+      <c r="I6" s="9" t="n">
+        <f aca="false">IFERROR(H6-A6,"")</f>
         <v>4</v>
       </c>
     </row>
@@ -2856,12 +2894,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A7,מקור!$L$2:$L$309,0)),"")</f>
         <v>34181.8</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A7,מקור!$L$2:$L$309,0)),"")</f>
+        <v>63211.5</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <f aca="false">IFERROR(E7/12*6,"")</f>
+        <v>31605.75</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <f aca="false">IFERROR(D7/F7-1,"")</f>
+        <v>0.0815057386709697</v>
+      </c>
+      <c r="H7" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A7,מקור!$L$2:$L$309,0)),"")</f>
         <v>3</v>
       </c>
-      <c r="F7" s="9" t="n">
-        <f aca="false">IFERROR(E7-A7,"")</f>
+      <c r="I7" s="9" t="n">
+        <f aca="false">IFERROR(H7-A7,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -2881,12 +2931,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A8,מקור!$L$2:$L$309,0)),"")</f>
         <v>34207.6</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A8,מקור!$L$2:$L$309,0)),"")</f>
+        <v>46442.7</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <f aca="false">IFERROR(E8/12*6,"")</f>
+        <v>23221.35</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <f aca="false">IFERROR(D8/F8-1,"")</f>
+        <v>0.473109875179522</v>
+      </c>
+      <c r="H8" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A8,מקור!$L$2:$L$309,0)),"")</f>
         <v>2</v>
       </c>
-      <c r="F8" s="9" t="n">
-        <f aca="false">IFERROR(E8-A8,"")</f>
+      <c r="I8" s="9" t="n">
+        <f aca="false">IFERROR(H8-A8,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -2906,12 +2968,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A9,מקור!$L$2:$L$309,0)),"")</f>
         <v>24091.9</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A9,מקור!$L$2:$L$309,0)),"")</f>
+        <v>50792.3</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <f aca="false">IFERROR(E9/12*6,"")</f>
+        <v>25396.15</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <f aca="false">IFERROR(D9/F9-1,"")</f>
+        <v>-0.0513562095041965</v>
+      </c>
+      <c r="H9" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A9,מקור!$L$2:$L$309,0)),"")</f>
         <v>9</v>
       </c>
-      <c r="F9" s="9" t="n">
-        <f aca="false">IFERROR(E9-A9,"")</f>
+      <c r="I9" s="9" t="n">
+        <f aca="false">IFERROR(H9-A9,"")</f>
         <v>4</v>
       </c>
     </row>
@@ -2931,12 +3005,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A10,מקור!$L$2:$L$309,0)),"")</f>
         <v>31106.1</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A10,מקור!$L$2:$L$309,0)),"")</f>
+        <v>51666.7</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <f aca="false">IFERROR(E10/12*6,"")</f>
+        <v>25833.35</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <f aca="false">IFERROR(D10/F10-1,"")</f>
+        <v>0.204106319931407</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A10,מקור!$L$2:$L$309,0)),"")</f>
         <v>5</v>
       </c>
-      <c r="F10" s="9" t="n">
-        <f aca="false">IFERROR(E10-A10,"")</f>
+      <c r="I10" s="9" t="n">
+        <f aca="false">IFERROR(H10-A10,"")</f>
         <v>-1</v>
       </c>
     </row>
@@ -2956,12 +3042,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A11,מקור!$L$2:$L$309,0)),"")</f>
         <v>21969.8</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A11,מקור!$L$2:$L$309,0)),"")</f>
+        <v>39005.8</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <f aca="false">IFERROR(E11/12*6,"")</f>
+        <v>19502.9</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <f aca="false">IFERROR(D11/F11-1,"")</f>
+        <v>0.126488881140753</v>
+      </c>
+      <c r="H11" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A11,מקור!$L$2:$L$309,0)),"")</f>
         <v>12</v>
       </c>
-      <c r="F11" s="9" t="n">
-        <f aca="false">IFERROR(E11-A11,"")</f>
+      <c r="I11" s="9" t="n">
+        <f aca="false">IFERROR(H11-A11,"")</f>
         <v>5</v>
       </c>
     </row>
@@ -2981,12 +3079,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A12,מקור!$L$2:$L$309,0)),"")</f>
         <v>25566.1</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A12,מקור!$L$2:$L$309,0)),"")</f>
+        <v>52586.4</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <f aca="false">IFERROR(E12/12*6,"")</f>
+        <v>26293.2</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <f aca="false">IFERROR(D12/F12-1,"")</f>
+        <v>-0.0276535377968448</v>
+      </c>
+      <c r="H12" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A12,מקור!$L$2:$L$309,0)),"")</f>
         <v>8</v>
       </c>
-      <c r="F12" s="9" t="n">
-        <f aca="false">IFERROR(E12-A12,"")</f>
+      <c r="I12" s="9" t="n">
+        <f aca="false">IFERROR(H12-A12,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -3006,12 +3116,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A13,מקור!$L$2:$L$309,0)),"")</f>
         <v>29916.7</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A13,מקור!$L$2:$L$309,0)),"")</f>
+        <v>56802.8</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <f aca="false">IFERROR(E13/12*6,"")</f>
+        <v>28401.4</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <f aca="false">IFERROR(D13/F13-1,"")</f>
+        <v>0.0533530037251684</v>
+      </c>
+      <c r="H13" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A13,מקור!$L$2:$L$309,0)),"")</f>
         <v>7</v>
       </c>
-      <c r="F13" s="9" t="n">
-        <f aca="false">IFERROR(E13-A13,"")</f>
+      <c r="I13" s="9" t="n">
+        <f aca="false">IFERROR(H13-A13,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -3031,12 +3153,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A14,מקור!$L$2:$L$309,0)),"")</f>
         <v>33328.8</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A14,מקור!$L$2:$L$309,0)),"")</f>
+        <v>58295.4</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <f aca="false">IFERROR(E14/12*6,"")</f>
+        <v>29147.7</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <f aca="false">IFERROR(D14/F14-1,"")</f>
+        <v>0.143445280416637</v>
+      </c>
+      <c r="H14" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A14,מקור!$L$2:$L$309,0)),"")</f>
         <v>4</v>
       </c>
-      <c r="F14" s="9" t="n">
-        <f aca="false">IFERROR(E14-A14,"")</f>
+      <c r="I14" s="9" t="n">
+        <f aca="false">IFERROR(H14-A14,"")</f>
         <v>-6</v>
       </c>
     </row>
@@ -3056,12 +3190,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A15,מקור!$L$2:$L$309,0)),"")</f>
         <v>22454.5</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A15,מקור!$L$2:$L$309,0)),"")</f>
+        <v>46557.9</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <f aca="false">IFERROR(E15/12*6,"")</f>
+        <v>23278.95</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <f aca="false">IFERROR(D15/F15-1,"")</f>
+        <v>-0.0354161162767221</v>
+      </c>
+      <c r="H15" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A15,מקור!$L$2:$L$309,0)),"")</f>
         <v>10</v>
       </c>
-      <c r="F15" s="9" t="n">
-        <f aca="false">IFERROR(E15-A15,"")</f>
+      <c r="I15" s="9" t="n">
+        <f aca="false">IFERROR(H15-A15,"")</f>
         <v>-1</v>
       </c>
     </row>
@@ -3081,12 +3227,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A16,מקור!$L$2:$L$309,0)),"")</f>
         <v>18434.6</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A16,מקור!$L$2:$L$309,0)),"")</f>
+        <v>36774.5</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <f aca="false">IFERROR(E16/12*6,"")</f>
+        <v>18387.25</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <f aca="false">IFERROR(D16/F16-1,"")</f>
+        <v>0.00257515397898001</v>
+      </c>
+      <c r="H16" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A16,מקור!$L$2:$L$309,0)),"")</f>
         <v>20</v>
       </c>
-      <c r="F16" s="9" t="n">
-        <f aca="false">IFERROR(E16-A16,"")</f>
+      <c r="I16" s="9" t="n">
+        <f aca="false">IFERROR(H16-A16,"")</f>
         <v>8</v>
       </c>
     </row>
@@ -3106,12 +3264,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A17,מקור!$L$2:$L$309,0)),"")</f>
         <v>21940.2</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A17,מקור!$L$2:$L$309,0)),"")</f>
+        <v>36086.4</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <f aca="false">IFERROR(E17/12*6,"")</f>
+        <v>18043.2</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <f aca="false">IFERROR(D17/F17-1,"")</f>
+        <v>0.21598164405427</v>
+      </c>
+      <c r="H17" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A17,מקור!$L$2:$L$309,0)),"")</f>
         <v>13</v>
       </c>
-      <c r="F17" s="9" t="n">
-        <f aca="false">IFERROR(E17-A17,"")</f>
+      <c r="I17" s="9" t="n">
+        <f aca="false">IFERROR(H17-A17,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -3131,12 +3301,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A18,מקור!$L$2:$L$309,0)),"")</f>
         <v>20373.4</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A18,מקור!$L$2:$L$309,0)),"")</f>
+        <v>35954.1</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <f aca="false">IFERROR(E18/12*6,"")</f>
+        <v>17977.05</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <f aca="false">IFERROR(D18/F18-1,"")</f>
+        <v>0.133300513710537</v>
+      </c>
+      <c r="H18" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A18,מקור!$L$2:$L$309,0)),"")</f>
         <v>15</v>
       </c>
-      <c r="F18" s="9" t="n">
-        <f aca="false">IFERROR(E18-A18,"")</f>
+      <c r="I18" s="9" t="n">
+        <f aca="false">IFERROR(H18-A18,"")</f>
         <v>1</v>
       </c>
     </row>
@@ -3156,12 +3338,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A19,מקור!$L$2:$L$309,0)),"")</f>
         <v>21728.9</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A19,מקור!$L$2:$L$309,0)),"")</f>
+        <v>40253.2</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <f aca="false">IFERROR(E19/12*6,"")</f>
+        <v>20126.6</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <f aca="false">IFERROR(D19/F19-1,"")</f>
+        <v>0.0796110619776815</v>
+      </c>
+      <c r="H19" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A19,מקור!$L$2:$L$309,0)),"")</f>
         <v>14</v>
       </c>
-      <c r="F19" s="9" t="n">
-        <f aca="false">IFERROR(E19-A19,"")</f>
+      <c r="I19" s="9" t="n">
+        <f aca="false">IFERROR(H19-A19,"")</f>
         <v>-1</v>
       </c>
     </row>
@@ -3181,12 +3375,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A20,מקור!$L$2:$L$309,0)),"")</f>
         <v>17265.6</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A20,מקור!$L$2:$L$309,0)),"")</f>
+        <v>29529.4</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <f aca="false">IFERROR(E20/12*6,"")</f>
+        <v>14764.7</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <f aca="false">IFERROR(D20/F20-1,"")</f>
+        <v>0.169383732822204</v>
+      </c>
+      <c r="H20" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A20,מקור!$L$2:$L$309,0)),"")</f>
         <v>23</v>
       </c>
-      <c r="F20" s="9" t="n">
-        <f aca="false">IFERROR(E20-A20,"")</f>
+      <c r="I20" s="9" t="n">
+        <f aca="false">IFERROR(H20-A20,"")</f>
         <v>7</v>
       </c>
     </row>
@@ -3206,12 +3412,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A21,מקור!$L$2:$L$309,0)),"")</f>
         <v>18749.5</v>
       </c>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A21,מקור!$L$2:$L$309,0)),"")</f>
+        <v>28337.4</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <f aca="false">IFERROR(E21/12*6,"")</f>
+        <v>14168.7</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <f aca="false">IFERROR(D21/F21-1,"")</f>
+        <v>0.323304184575861</v>
+      </c>
+      <c r="H21" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A21,מקור!$L$2:$L$309,0)),"")</f>
         <v>19</v>
       </c>
-      <c r="F21" s="9" t="n">
-        <f aca="false">IFERROR(E21-A21,"")</f>
+      <c r="I21" s="9" t="n">
+        <f aca="false">IFERROR(H21-A21,"")</f>
         <v>2</v>
       </c>
     </row>
@@ -3231,12 +3449,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A22,מקור!$L$2:$L$309,0)),"")</f>
         <v>22141.7</v>
       </c>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A22,מקור!$L$2:$L$309,0)),"")</f>
+        <v>42012.2</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <f aca="false">IFERROR(E22/12*6,"")</f>
+        <v>21006.1</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <f aca="false">IFERROR(D22/F22-1,"")</f>
+        <v>0.0540604871918158</v>
+      </c>
+      <c r="H22" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A22,מקור!$L$2:$L$309,0)),"")</f>
         <v>11</v>
       </c>
-      <c r="F22" s="9" t="n">
-        <f aca="false">IFERROR(E22-A22,"")</f>
+      <c r="I22" s="9" t="n">
+        <f aca="false">IFERROR(H22-A22,"")</f>
         <v>-7</v>
       </c>
     </row>
@@ -3256,12 +3486,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A23,מקור!$L$2:$L$309,0)),"")</f>
         <v>19760.5</v>
       </c>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A23,מקור!$L$2:$L$309,0)),"")</f>
+        <v>37059</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <f aca="false">IFERROR(E23/12*6,"")</f>
+        <v>18529.5</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <f aca="false">IFERROR(D23/F23-1,"")</f>
+        <v>0.0664346042796622</v>
+      </c>
+      <c r="H23" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A23,מקור!$L$2:$L$309,0)),"")</f>
         <v>16</v>
       </c>
-      <c r="F23" s="9" t="n">
-        <f aca="false">IFERROR(E23-A23,"")</f>
+      <c r="I23" s="9" t="n">
+        <f aca="false">IFERROR(H23-A23,"")</f>
         <v>-3</v>
       </c>
     </row>
@@ -3281,12 +3523,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A24,מקור!$L$2:$L$309,0)),"")</f>
         <v>19715.9</v>
       </c>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A24,מקור!$L$2:$L$309,0)),"")</f>
+        <v>45291.6</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <f aca="false">IFERROR(E24/12*6,"")</f>
+        <v>22645.8</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <f aca="false">IFERROR(D24/F24-1,"")</f>
+        <v>-0.129379399270505</v>
+      </c>
+      <c r="H24" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A24,מקור!$L$2:$L$309,0)),"")</f>
         <v>17</v>
       </c>
-      <c r="F24" s="9" t="n">
-        <f aca="false">IFERROR(E24-A24,"")</f>
+      <c r="I24" s="9" t="n">
+        <f aca="false">IFERROR(H24-A24,"")</f>
         <v>-3</v>
       </c>
     </row>
@@ -3306,12 +3560,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A25,מקור!$L$2:$L$309,0)),"")</f>
         <v>17795.5</v>
       </c>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A25,מקור!$L$2:$L$309,0)),"")</f>
+        <v>33328.1</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <f aca="false">IFERROR(E25/12*6,"")</f>
+        <v>16664.05</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <f aca="false">IFERROR(D25/F25-1,"")</f>
+        <v>0.0678976599326095</v>
+      </c>
+      <c r="H25" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A25,מקור!$L$2:$L$309,0)),"")</f>
         <v>21</v>
       </c>
-      <c r="F25" s="9" t="n">
-        <f aca="false">IFERROR(E25-A25,"")</f>
+      <c r="I25" s="9" t="n">
+        <f aca="false">IFERROR(H25-A25,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -3331,12 +3597,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A26,מקור!$L$2:$L$309,0)),"")</f>
         <v>14413.6</v>
       </c>
-      <c r="E26" s="5" t="n">
+      <c r="E26" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A26,מקור!$L$2:$L$309,0)),"")</f>
+        <v>28455.3</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <f aca="false">IFERROR(E26/12*6,"")</f>
+        <v>14227.65</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <f aca="false">IFERROR(D26/F26-1,"")</f>
+        <v>0.0130696214764912</v>
+      </c>
+      <c r="H26" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A26,מקור!$L$2:$L$309,0)),"")</f>
         <v>25</v>
       </c>
-      <c r="F26" s="9" t="n">
-        <f aca="false">IFERROR(E26-A26,"")</f>
+      <c r="I26" s="9" t="n">
+        <f aca="false">IFERROR(H26-A26,"")</f>
         <v>3</v>
       </c>
     </row>
@@ -3356,12 +3634,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A27,מקור!$L$2:$L$309,0)),"")</f>
         <v>19057.1</v>
       </c>
-      <c r="E27" s="5" t="n">
+      <c r="E27" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A27,מקור!$L$2:$L$309,0)),"")</f>
+        <v>37677.9</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <f aca="false">IFERROR(E27/12*6,"")</f>
+        <v>18838.95</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <f aca="false">IFERROR(D27/F27-1,"")</f>
+        <v>0.0115797324160847</v>
+      </c>
+      <c r="H27" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A27,מקור!$L$2:$L$309,0)),"")</f>
         <v>18</v>
       </c>
-      <c r="F27" s="9" t="n">
-        <f aca="false">IFERROR(E27-A27,"")</f>
+      <c r="I27" s="9" t="n">
+        <f aca="false">IFERROR(H27-A27,"")</f>
         <v>-5</v>
       </c>
     </row>
@@ -3381,12 +3671,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A28,מקור!$L$2:$L$309,0)),"")</f>
         <v>13139.5</v>
       </c>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A28,מקור!$L$2:$L$309,0)),"")</f>
+        <v>30442.7</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <f aca="false">IFERROR(E28/12*6,"")</f>
+        <v>15221.35</v>
+      </c>
+      <c r="G28" s="7" t="n">
+        <f aca="false">IFERROR(D28/F28-1,"")</f>
+        <v>-0.136771705532032</v>
+      </c>
+      <c r="H28" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A28,מקור!$L$2:$L$309,0)),"")</f>
         <v>31</v>
       </c>
-      <c r="F28" s="9" t="n">
-        <f aca="false">IFERROR(E28-A28,"")</f>
+      <c r="I28" s="9" t="n">
+        <f aca="false">IFERROR(H28-A28,"")</f>
         <v>7</v>
       </c>
     </row>
@@ -3406,12 +3708,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A29,מקור!$L$2:$L$309,0)),"")</f>
         <v>15060.5</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A29,מקור!$L$2:$L$309,0)),"")</f>
+        <v>29506.2</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <f aca="false">IFERROR(E29/12*6,"")</f>
+        <v>14753.1</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <f aca="false">IFERROR(D29/F29-1,"")</f>
+        <v>0.0208362988117752</v>
+      </c>
+      <c r="H29" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A29,מקור!$L$2:$L$309,0)),"")</f>
         <v>24</v>
       </c>
-      <c r="F29" s="9" t="n">
-        <f aca="false">IFERROR(E29-A29,"")</f>
+      <c r="I29" s="9" t="n">
+        <f aca="false">IFERROR(H29-A29,"")</f>
         <v>-1</v>
       </c>
     </row>
@@ -3431,12 +3745,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A30,מקור!$L$2:$L$309,0)),"")</f>
         <v>17541.3</v>
       </c>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A30,מקור!$L$2:$L$309,0)),"")</f>
+        <v>28284.4</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <f aca="false">IFERROR(E30/12*6,"")</f>
+        <v>14142.2</v>
+      </c>
+      <c r="G30" s="7" t="n">
+        <f aca="false">IFERROR(D30/F30-1,"")</f>
+        <v>0.240351571891219</v>
+      </c>
+      <c r="H30" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A30,מקור!$L$2:$L$309,0)),"")</f>
         <v>22</v>
       </c>
-      <c r="F30" s="9" t="n">
-        <f aca="false">IFERROR(E30-A30,"")</f>
+      <c r="I30" s="9" t="n">
+        <f aca="false">IFERROR(H30-A30,"")</f>
         <v>-4</v>
       </c>
     </row>
@@ -3456,12 +3782,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A31,מקור!$L$2:$L$309,0)),"")</f>
         <v>13789.2</v>
       </c>
-      <c r="E31" s="5" t="n">
+      <c r="E31" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A31,מקור!$L$2:$L$309,0)),"")</f>
+        <v>23706.5</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <f aca="false">IFERROR(E31/12*6,"")</f>
+        <v>11853.25</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <f aca="false">IFERROR(D31/F31-1,"")</f>
+        <v>0.163326513825322</v>
+      </c>
+      <c r="H31" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A31,מקור!$L$2:$L$309,0)),"")</f>
         <v>28</v>
       </c>
-      <c r="F31" s="9" t="n">
-        <f aca="false">IFERROR(E31-A31,"")</f>
+      <c r="I31" s="9" t="n">
+        <f aca="false">IFERROR(H31-A31,"")</f>
         <v>1</v>
       </c>
     </row>
@@ -3481,12 +3819,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A32,מקור!$L$2:$L$309,0)),"")</f>
         <v>10738.9</v>
       </c>
-      <c r="E32" s="5" t="n">
+      <c r="E32" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A32,מקור!$L$2:$L$309,0)),"")</f>
+        <v>27958.3</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <f aca="false">IFERROR(E32/12*6,"")</f>
+        <v>13979.15</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <f aca="false">IFERROR(D32/F32-1,"")</f>
+        <v>-0.231791632538459</v>
+      </c>
+      <c r="H32" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A32,מקור!$L$2:$L$309,0)),"")</f>
         <v>40</v>
       </c>
-      <c r="F32" s="9" t="n">
-        <f aca="false">IFERROR(E32-A32,"")</f>
+      <c r="I32" s="9" t="n">
+        <f aca="false">IFERROR(H32-A32,"")</f>
         <v>12</v>
       </c>
     </row>
@@ -3506,12 +3856,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A33,מקור!$L$2:$L$309,0)),"")</f>
         <v>14027.5</v>
       </c>
-      <c r="E33" s="5" t="n">
+      <c r="E33" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A33,מקור!$L$2:$L$309,0)),"")</f>
+        <v>28961</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <f aca="false">IFERROR(E33/12*6,"")</f>
+        <v>14480.5</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <f aca="false">IFERROR(D33/F33-1,"")</f>
+        <v>-0.0312834501571079</v>
+      </c>
+      <c r="H33" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A33,מקור!$L$2:$L$309,0)),"")</f>
         <v>27</v>
       </c>
-      <c r="F33" s="9" t="n">
-        <f aca="false">IFERROR(E33-A33,"")</f>
+      <c r="I33" s="9" t="n">
+        <f aca="false">IFERROR(H33-A33,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -3531,12 +3893,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A34,מקור!$L$2:$L$309,0)),"")</f>
         <v>9066.9</v>
       </c>
-      <c r="E34" s="5" t="n">
+      <c r="E34" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A34,מקור!$L$2:$L$309,0)),"")</f>
+        <v>29751.8</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <f aca="false">IFERROR(E34/12*6,"")</f>
+        <v>14875.9</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <f aca="false">IFERROR(D34/F34-1,"")</f>
+        <v>-0.390497381671025</v>
+      </c>
+      <c r="H34" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A34,מקור!$L$2:$L$309,0)),"")</f>
         <v>46</v>
       </c>
-      <c r="F34" s="9" t="n">
-        <f aca="false">IFERROR(E34-A34,"")</f>
+      <c r="I34" s="9" t="n">
+        <f aca="false">IFERROR(H34-A34,"")</f>
         <v>16</v>
       </c>
     </row>
@@ -3556,12 +3930,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A35,מקור!$L$2:$L$309,0)),"")</f>
         <v>12396.5</v>
       </c>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A35,מקור!$L$2:$L$309,0)),"")</f>
+        <v>24221.5</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <f aca="false">IFERROR(E35/12*6,"")</f>
+        <v>12110.75</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <f aca="false">IFERROR(D35/F35-1,"")</f>
+        <v>0.023594740210144</v>
+      </c>
+      <c r="H35" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A35,מקור!$L$2:$L$309,0)),"")</f>
         <v>34</v>
       </c>
-      <c r="F35" s="9" t="n">
-        <f aca="false">IFERROR(E35-A35,"")</f>
+      <c r="I35" s="9" t="n">
+        <f aca="false">IFERROR(H35-A35,"")</f>
         <v>3</v>
       </c>
     </row>
@@ -3581,12 +3967,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A36,מקור!$L$2:$L$309,0)),"")</f>
         <v>11554.9</v>
       </c>
-      <c r="E36" s="5" t="n">
+      <c r="E36" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A36,מקור!$L$2:$L$309,0)),"")</f>
+        <v>20992.4</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <f aca="false">IFERROR(E36/12*6,"")</f>
+        <v>10496.2</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <f aca="false">IFERROR(D36/F36-1,"")</f>
+        <v>0.100865074979516</v>
+      </c>
+      <c r="H36" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A36,מקור!$L$2:$L$309,0)),"")</f>
         <v>36</v>
       </c>
-      <c r="F36" s="9" t="n">
-        <f aca="false">IFERROR(E36-A36,"")</f>
+      <c r="I36" s="9" t="n">
+        <f aca="false">IFERROR(H36-A36,"")</f>
         <v>4</v>
       </c>
     </row>
@@ -3606,12 +4004,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A37,מקור!$L$2:$L$309,0)),"")</f>
         <v>14054.4</v>
       </c>
-      <c r="E37" s="5" t="n">
+      <c r="E37" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A37,מקור!$L$2:$L$309,0)),"")</f>
+        <v>29037.3</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <f aca="false">IFERROR(E37/12*6,"")</f>
+        <v>14518.65</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <f aca="false">IFERROR(D37/F37-1,"")</f>
+        <v>-0.0319761134816254</v>
+      </c>
+      <c r="H37" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A37,מקור!$L$2:$L$309,0)),"")</f>
         <v>26</v>
       </c>
-      <c r="F37" s="9" t="n">
-        <f aca="false">IFERROR(E37-A37,"")</f>
+      <c r="I37" s="9" t="n">
+        <f aca="false">IFERROR(H37-A37,"")</f>
         <v>-7</v>
       </c>
     </row>
@@ -3631,12 +4041,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A38,מקור!$L$2:$L$309,0)),"")</f>
         <v>12889.3</v>
       </c>
-      <c r="E38" s="5" t="n">
+      <c r="E38" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A38,מקור!$L$2:$L$309,0)),"")</f>
+        <v>13546.6</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <f aca="false">IFERROR(E38/12*6,"")</f>
+        <v>6773.3</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <f aca="false">IFERROR(D38/F38-1,"")</f>
+        <v>0.902957199592517</v>
+      </c>
+      <c r="H38" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A38,מקור!$L$2:$L$309,0)),"")</f>
         <v>32</v>
       </c>
-      <c r="F38" s="9" t="n">
-        <f aca="false">IFERROR(E38-A38,"")</f>
+      <c r="I38" s="9" t="n">
+        <f aca="false">IFERROR(H38-A38,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -3656,12 +4078,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A39,מקור!$L$2:$L$309,0)),"")</f>
         <v>11597.1</v>
       </c>
-      <c r="E39" s="5" t="n">
+      <c r="E39" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A39,מקור!$L$2:$L$309,0)),"")</f>
+        <v>22838.4</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <f aca="false">IFERROR(E39/12*6,"")</f>
+        <v>11419.2</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <f aca="false">IFERROR(D39/F39-1,"")</f>
+        <v>0.0155790248003362</v>
+      </c>
+      <c r="H39" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A39,מקור!$L$2:$L$309,0)),"")</f>
         <v>35</v>
       </c>
-      <c r="F39" s="9" t="n">
-        <f aca="false">IFERROR(E39-A39,"")</f>
+      <c r="I39" s="9" t="n">
+        <f aca="false">IFERROR(H39-A39,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -3681,12 +4115,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A40,מקור!$L$2:$L$309,0)),"")</f>
         <v>13513.8</v>
       </c>
-      <c r="E40" s="5" t="n">
+      <c r="E40" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A40,מקור!$L$2:$L$309,0)),"")</f>
+        <v>28096.6</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <f aca="false">IFERROR(E40/12*6,"")</f>
+        <v>14048.3</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <f aca="false">IFERROR(D40/F40-1,"")</f>
+        <v>-0.0380473082152288</v>
+      </c>
+      <c r="H40" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A40,מקור!$L$2:$L$309,0)),"")</f>
         <v>29</v>
       </c>
-      <c r="F40" s="9" t="n">
-        <f aca="false">IFERROR(E40-A40,"")</f>
+      <c r="I40" s="9" t="n">
+        <f aca="false">IFERROR(H40-A40,"")</f>
         <v>-7</v>
       </c>
     </row>
@@ -3706,12 +4152,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A41,מקור!$L$2:$L$309,0)),"")</f>
         <v>12807.3</v>
       </c>
-      <c r="E41" s="5" t="n">
+      <c r="E41" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A41,מקור!$L$2:$L$309,0)),"")</f>
+        <v>26317.6</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <f aca="false">IFERROR(E41/12*6,"")</f>
+        <v>13158.8</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <f aca="false">IFERROR(D41/F41-1,"")</f>
+        <v>-0.0267121622032405</v>
+      </c>
+      <c r="H41" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A41,מקור!$L$2:$L$309,0)),"")</f>
         <v>33</v>
       </c>
-      <c r="F41" s="9" t="n">
-        <f aca="false">IFERROR(E41-A41,"")</f>
+      <c r="I41" s="9" t="n">
+        <f aca="false">IFERROR(H41-A41,"")</f>
         <v>-4</v>
       </c>
     </row>
@@ -3731,12 +4189,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A42,מקור!$L$2:$L$309,0)),"")</f>
         <v>13484.7</v>
       </c>
-      <c r="E42" s="5" t="n">
+      <c r="E42" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A42,מקור!$L$2:$L$309,0)),"")</f>
+        <v>28489.4</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <f aca="false">IFERROR(E42/12*6,"")</f>
+        <v>14244.7</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <f aca="false">IFERROR(D42/F42-1,"")</f>
+        <v>-0.053353176971084</v>
+      </c>
+      <c r="H42" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A42,מקור!$L$2:$L$309,0)),"")</f>
         <v>30</v>
       </c>
-      <c r="F42" s="9" t="n">
-        <f aca="false">IFERROR(E42-A42,"")</f>
+      <c r="I42" s="9" t="n">
+        <f aca="false">IFERROR(H42-A42,"")</f>
         <v>-8</v>
       </c>
     </row>
@@ -3756,12 +4226,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A43,מקור!$L$2:$L$309,0)),"")</f>
         <v>11342.2</v>
       </c>
-      <c r="E43" s="5" t="n">
+      <c r="E43" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A43,מקור!$L$2:$L$309,0)),"")</f>
+        <v>23771</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <f aca="false">IFERROR(E43/12*6,"")</f>
+        <v>11885.5</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <f aca="false">IFERROR(D43/F43-1,"")</f>
+        <v>-0.0457111606579445</v>
+      </c>
+      <c r="H43" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A43,מקור!$L$2:$L$309,0)),"")</f>
         <v>37</v>
       </c>
-      <c r="F43" s="9" t="n">
-        <f aca="false">IFERROR(E43-A43,"")</f>
+      <c r="I43" s="9" t="n">
+        <f aca="false">IFERROR(H43-A43,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -3781,12 +4263,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A44,מקור!$L$2:$L$309,0)),"")</f>
         <v>11193</v>
       </c>
-      <c r="E44" s="5" t="n">
+      <c r="E44" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A44,מקור!$L$2:$L$309,0)),"")</f>
+        <v>25344.6</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <f aca="false">IFERROR(E44/12*6,"")</f>
+        <v>12672.3</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <f aca="false">IFERROR(D44/F44-1,"")</f>
+        <v>-0.116734925783007</v>
+      </c>
+      <c r="H44" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A44,מקור!$L$2:$L$309,0)),"")</f>
         <v>38</v>
       </c>
-      <c r="F44" s="9" t="n">
-        <f aca="false">IFERROR(E44-A44,"")</f>
+      <c r="I44" s="9" t="n">
+        <f aca="false">IFERROR(H44-A44,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -3806,12 +4300,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A45,מקור!$L$2:$L$309,0)),"")</f>
         <v>9529.3</v>
       </c>
-      <c r="E45" s="5" t="n">
+      <c r="E45" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A45,מקור!$L$2:$L$309,0)),"")</f>
+        <v>19456</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <f aca="false">IFERROR(E45/12*6,"")</f>
+        <v>9728</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <f aca="false">IFERROR(D45/F45-1,"")</f>
+        <v>-0.0204255756578948</v>
+      </c>
+      <c r="H45" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A45,מקור!$L$2:$L$309,0)),"")</f>
         <v>43</v>
       </c>
-      <c r="F45" s="9" t="n">
-        <f aca="false">IFERROR(E45-A45,"")</f>
+      <c r="I45" s="9" t="n">
+        <f aca="false">IFERROR(H45-A45,"")</f>
         <v>2</v>
       </c>
     </row>
@@ -3831,12 +4337,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A46,מקור!$L$2:$L$309,0)),"")</f>
         <v>7642.2</v>
       </c>
-      <c r="E46" s="5" t="n">
+      <c r="E46" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A46,מקור!$L$2:$L$309,0)),"")</f>
+        <v>14420.5</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <f aca="false">IFERROR(E46/12*6,"")</f>
+        <v>7210.25</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <f aca="false">IFERROR(D46/F46-1,"")</f>
+        <v>0.0599077701882735</v>
+      </c>
+      <c r="H46" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A46,מקור!$L$2:$L$309,0)),"")</f>
         <v>48</v>
       </c>
-      <c r="F46" s="9" t="n">
-        <f aca="false">IFERROR(E46-A46,"")</f>
+      <c r="I46" s="9" t="n">
+        <f aca="false">IFERROR(H46-A46,"")</f>
         <v>6</v>
       </c>
     </row>
@@ -3856,12 +4374,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A47,מקור!$L$2:$L$309,0)),"")</f>
         <v>8075.6</v>
       </c>
-      <c r="E47" s="5" t="n">
+      <c r="E47" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A47,מקור!$L$2:$L$309,0)),"")</f>
+        <v>13370.5</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <f aca="false">IFERROR(E47/12*6,"")</f>
+        <v>6685.25</v>
+      </c>
+      <c r="G47" s="7" t="n">
+        <f aca="false">IFERROR(D47/F47-1,"")</f>
+        <v>0.207972775887215</v>
+      </c>
+      <c r="H47" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A47,מקור!$L$2:$L$309,0)),"")</f>
         <v>47</v>
       </c>
-      <c r="F47" s="9" t="n">
-        <f aca="false">IFERROR(E47-A47,"")</f>
+      <c r="I47" s="9" t="n">
+        <f aca="false">IFERROR(H47-A47,"")</f>
         <v>4</v>
       </c>
     </row>
@@ -3881,12 +4411,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A48,מקור!$L$2:$L$309,0)),"")</f>
         <v>6409.1</v>
       </c>
-      <c r="E48" s="5" t="n">
+      <c r="E48" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A48,מקור!$L$2:$L$309,0)),"")</f>
+        <v>15834.2</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <f aca="false">IFERROR(E48/12*6,"")</f>
+        <v>7917.1</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <f aca="false">IFERROR(D48/F48-1,"")</f>
+        <v>-0.190473784592843</v>
+      </c>
+      <c r="H48" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A48,מקור!$L$2:$L$309,0)),"")</f>
         <v>53</v>
       </c>
-      <c r="F48" s="9" t="n">
-        <f aca="false">IFERROR(E48-A48,"")</f>
+      <c r="I48" s="9" t="n">
+        <f aca="false">IFERROR(H48-A48,"")</f>
         <v>9</v>
       </c>
     </row>
@@ -3906,12 +4448,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A49,מקור!$L$2:$L$309,0)),"")</f>
         <v>9090.1</v>
       </c>
-      <c r="E49" s="5" t="n">
+      <c r="E49" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A49,מקור!$L$2:$L$309,0)),"")</f>
+        <v>19282.8</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <f aca="false">IFERROR(E49/12*6,"")</f>
+        <v>9641.4</v>
+      </c>
+      <c r="G49" s="7" t="n">
+        <f aca="false">IFERROR(D49/F49-1,"")</f>
+        <v>-0.0571804924596012</v>
+      </c>
+      <c r="H49" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A49,מקור!$L$2:$L$309,0)),"")</f>
         <v>45</v>
       </c>
-      <c r="F49" s="9" t="n">
-        <f aca="false">IFERROR(E49-A49,"")</f>
+      <c r="I49" s="9" t="n">
+        <f aca="false">IFERROR(H49-A49,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -3931,12 +4485,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A50,מקור!$L$2:$L$309,0)),"")</f>
         <v>9835.3</v>
       </c>
-      <c r="E50" s="5" t="n">
+      <c r="E50" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A50,מקור!$L$2:$L$309,0)),"")</f>
+        <v>19470.7</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <f aca="false">IFERROR(E50/12*6,"")</f>
+        <v>9735.35</v>
+      </c>
+      <c r="G50" s="7" t="n">
+        <f aca="false">IFERROR(D50/F50-1,"")</f>
+        <v>0.0102667084388337</v>
+      </c>
+      <c r="H50" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A50,מקור!$L$2:$L$309,0)),"")</f>
         <v>42</v>
       </c>
-      <c r="F50" s="9" t="n">
-        <f aca="false">IFERROR(E50-A50,"")</f>
+      <c r="I50" s="9" t="n">
+        <f aca="false">IFERROR(H50-A50,"")</f>
         <v>-4</v>
       </c>
     </row>
@@ -3956,12 +4522,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A51,מקור!$L$2:$L$309,0)),"")</f>
         <v>5519.3</v>
       </c>
-      <c r="E51" s="5" t="n">
+      <c r="E51" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A51,מקור!$L$2:$L$309,0)),"")</f>
+        <v>15986</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <f aca="false">IFERROR(E51/12*6,"")</f>
+        <v>7993</v>
+      </c>
+      <c r="G51" s="7" t="n">
+        <f aca="false">IFERROR(D51/F51-1,"")</f>
+        <v>-0.30948329788565</v>
+      </c>
+      <c r="H51" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A51,מקור!$L$2:$L$309,0)),"")</f>
         <v>57</v>
       </c>
-      <c r="F51" s="9" t="n">
-        <f aca="false">IFERROR(E51-A51,"")</f>
+      <c r="I51" s="9" t="n">
+        <f aca="false">IFERROR(H51-A51,"")</f>
         <v>10</v>
       </c>
     </row>
@@ -3981,12 +4559,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A52,מקור!$L$2:$L$309,0)),"")</f>
         <v>9168.6</v>
       </c>
-      <c r="E52" s="5" t="n">
+      <c r="E52" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A52,מקור!$L$2:$L$309,0)),"")</f>
+        <v>19476.1</v>
+      </c>
+      <c r="F52" s="6" t="n">
+        <f aca="false">IFERROR(E52/12*6,"")</f>
+        <v>9738.05</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <f aca="false">IFERROR(D52/F52-1,"")</f>
+        <v>-0.0584767997699743</v>
+      </c>
+      <c r="H52" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A52,מקור!$L$2:$L$309,0)),"")</f>
         <v>44</v>
       </c>
-      <c r="F52" s="9" t="n">
-        <f aca="false">IFERROR(E52-A52,"")</f>
+      <c r="I52" s="9" t="n">
+        <f aca="false">IFERROR(H52-A52,"")</f>
         <v>-4</v>
       </c>
     </row>
@@ -4006,12 +4596,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A53,מקור!$L$2:$L$309,0)),"")</f>
         <v>10901.1</v>
       </c>
-      <c r="E53" s="5" t="n">
+      <c r="E53" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A53,מקור!$L$2:$L$309,0)),"")</f>
+        <v>22230.3</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <f aca="false">IFERROR(E53/12*6,"")</f>
+        <v>11115.15</v>
+      </c>
+      <c r="G53" s="7" t="n">
+        <f aca="false">IFERROR(D53/F53-1,"")</f>
+        <v>-0.0192574998987868</v>
+      </c>
+      <c r="H53" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A53,מקור!$L$2:$L$309,0)),"")</f>
         <v>39</v>
       </c>
-      <c r="F53" s="9" t="n">
-        <f aca="false">IFERROR(E53-A53,"")</f>
+      <c r="I53" s="9" t="n">
+        <f aca="false">IFERROR(H53-A53,"")</f>
         <v>-10</v>
       </c>
     </row>
@@ -4031,12 +4633,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A54,מקור!$L$2:$L$309,0)),"")</f>
         <v>6840.4</v>
       </c>
-      <c r="E54" s="5" t="n">
+      <c r="E54" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A54,מקור!$L$2:$L$309,0)),"")</f>
+        <v>13276.6</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <f aca="false">IFERROR(E54/12*6,"")</f>
+        <v>6638.3</v>
+      </c>
+      <c r="G54" s="7" t="n">
+        <f aca="false">IFERROR(D54/F54-1,"")</f>
+        <v>0.0304445415241852</v>
+      </c>
+      <c r="H54" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A54,מקור!$L$2:$L$309,0)),"")</f>
         <v>52</v>
       </c>
-      <c r="F54" s="9" t="n">
-        <f aca="false">IFERROR(E54-A54,"")</f>
+      <c r="I54" s="9" t="n">
+        <f aca="false">IFERROR(H54-A54,"")</f>
         <v>2</v>
       </c>
     </row>
@@ -4056,12 +4670,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A55,מקור!$L$2:$L$309,0)),"")</f>
         <v>7071.2</v>
       </c>
-      <c r="E55" s="5" t="n">
+      <c r="E55" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A55,מקור!$L$2:$L$309,0)),"")</f>
+        <v>12606.8</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <f aca="false">IFERROR(E55/12*6,"")</f>
+        <v>6303.4</v>
+      </c>
+      <c r="G55" s="7" t="n">
+        <f aca="false">IFERROR(D55/F55-1,"")</f>
+        <v>0.121807278611543</v>
+      </c>
+      <c r="H55" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A55,מקור!$L$2:$L$309,0)),"")</f>
         <v>51</v>
       </c>
-      <c r="F55" s="9" t="n">
-        <f aca="false">IFERROR(E55-A55,"")</f>
+      <c r="I55" s="9" t="n">
+        <f aca="false">IFERROR(H55-A55,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -4081,12 +4707,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A56,מקור!$L$2:$L$309,0)),"")</f>
         <v>7097.5</v>
       </c>
-      <c r="E56" s="5" t="n">
+      <c r="E56" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A56,מקור!$L$2:$L$309,0)),"")</f>
+        <v>18474.4</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <f aca="false">IFERROR(E56/12*6,"")</f>
+        <v>9237.2</v>
+      </c>
+      <c r="G56" s="7" t="n">
+        <f aca="false">IFERROR(D56/F56-1,"")</f>
+        <v>-0.231639457844368</v>
+      </c>
+      <c r="H56" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A56,מקור!$L$2:$L$309,0)),"")</f>
         <v>50</v>
       </c>
-      <c r="F56" s="9" t="n">
-        <f aca="false">IFERROR(E56-A56,"")</f>
+      <c r="I56" s="9" t="n">
+        <f aca="false">IFERROR(H56-A56,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -4106,12 +4744,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A57,מקור!$L$2:$L$309,0)),"")</f>
         <v>7577.1</v>
       </c>
-      <c r="E57" s="5" t="n">
+      <c r="E57" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A57,מקור!$L$2:$L$309,0)),"")</f>
+        <v>31858.7</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <f aca="false">IFERROR(E57/12*6,"")</f>
+        <v>15929.35</v>
+      </c>
+      <c r="G57" s="7" t="n">
+        <f aca="false">IFERROR(D57/F57-1,"")</f>
+        <v>-0.524330873513357</v>
+      </c>
+      <c r="H57" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A57,מקור!$L$2:$L$309,0)),"")</f>
         <v>49</v>
       </c>
-      <c r="F57" s="9" t="n">
-        <f aca="false">IFERROR(E57-A57,"")</f>
+      <c r="I57" s="9" t="n">
+        <f aca="false">IFERROR(H57-A57,"")</f>
         <v>-4</v>
       </c>
     </row>
@@ -4131,12 +4781,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A58,מקור!$L$2:$L$309,0)),"")</f>
         <v>4713.3</v>
       </c>
-      <c r="E58" s="5" t="n">
+      <c r="E58" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A58,מקור!$L$2:$L$309,0)),"")</f>
+        <v>11455.5</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <f aca="false">IFERROR(E58/12*6,"")</f>
+        <v>5727.75</v>
+      </c>
+      <c r="G58" s="7" t="n">
+        <f aca="false">IFERROR(D58/F58-1,"")</f>
+        <v>-0.177111431190258</v>
+      </c>
+      <c r="H58" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A58,מקור!$L$2:$L$309,0)),"")</f>
         <v>60</v>
       </c>
-      <c r="F58" s="9" t="n">
-        <f aca="false">IFERROR(E58-A58,"")</f>
+      <c r="I58" s="9" t="n">
+        <f aca="false">IFERROR(H58-A58,"")</f>
         <v>6</v>
       </c>
     </row>
@@ -4156,12 +4818,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A59,מקור!$L$2:$L$309,0)),"")</f>
         <v>10094.1</v>
       </c>
-      <c r="E59" s="5" t="n">
+      <c r="E59" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A59,מקור!$L$2:$L$309,0)),"")</f>
+        <v>17473.5</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <f aca="false">IFERROR(E59/12*6,"")</f>
+        <v>8736.75</v>
+      </c>
+      <c r="G59" s="7" t="n">
+        <f aca="false">IFERROR(D59/F59-1,"")</f>
+        <v>0.155360975191004</v>
+      </c>
+      <c r="H59" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A59,מקור!$L$2:$L$309,0)),"")</f>
         <v>41</v>
       </c>
-      <c r="F59" s="9" t="n">
-        <f aca="false">IFERROR(E59-A59,"")</f>
+      <c r="I59" s="9" t="n">
+        <f aca="false">IFERROR(H59-A59,"")</f>
         <v>-14</v>
       </c>
     </row>
@@ -4181,12 +4855,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A60,מקור!$L$2:$L$309,0)),"")</f>
         <v>5815.8</v>
       </c>
-      <c r="E60" s="5" t="n">
+      <c r="E60" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A60,מקור!$L$2:$L$309,0)),"")</f>
+        <v>12988</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <f aca="false">IFERROR(E60/12*6,"")</f>
+        <v>6494</v>
+      </c>
+      <c r="G60" s="7" t="n">
+        <f aca="false">IFERROR(D60/F60-1,"")</f>
+        <v>-0.104434862950416</v>
+      </c>
+      <c r="H60" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A60,מקור!$L$2:$L$309,0)),"")</f>
         <v>55</v>
       </c>
-      <c r="F60" s="9" t="n">
-        <f aca="false">IFERROR(E60-A60,"")</f>
+      <c r="I60" s="9" t="n">
+        <f aca="false">IFERROR(H60-A60,"")</f>
         <v>-1</v>
       </c>
     </row>
@@ -4206,12 +4892,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A61,מקור!$L$2:$L$309,0)),"")</f>
         <v>5259.1</v>
       </c>
-      <c r="E61" s="5" t="n">
+      <c r="E61" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A61,מקור!$L$2:$L$309,0)),"")</f>
+        <v>17310.2</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <f aca="false">IFERROR(E61/12*6,"")</f>
+        <v>8655.1</v>
+      </c>
+      <c r="G61" s="7" t="n">
+        <f aca="false">IFERROR(D61/F61-1,"")</f>
+        <v>-0.3923698166399</v>
+      </c>
+      <c r="H61" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A61,מקור!$L$2:$L$309,0)),"")</f>
         <v>58</v>
       </c>
-      <c r="F61" s="9" t="n">
-        <f aca="false">IFERROR(E61-A61,"")</f>
+      <c r="I61" s="9" t="n">
+        <f aca="false">IFERROR(H61-A61,"")</f>
         <v>1</v>
       </c>
     </row>
@@ -4231,12 +4929,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A62,מקור!$L$2:$L$309,0)),"")</f>
         <v>6204.2</v>
       </c>
-      <c r="E62" s="5" t="n">
+      <c r="E62" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A62,מקור!$L$2:$L$309,0)),"")</f>
+        <v>11348.6</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <f aca="false">IFERROR(E62/12*6,"")</f>
+        <v>5674.3</v>
+      </c>
+      <c r="G62" s="7" t="n">
+        <f aca="false">IFERROR(D62/F62-1,"")</f>
+        <v>0.0933859683132721</v>
+      </c>
+      <c r="H62" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A62,מקור!$L$2:$L$309,0)),"")</f>
         <v>54</v>
       </c>
-      <c r="F62" s="9" t="n">
-        <f aca="false">IFERROR(E62-A62,"")</f>
+      <c r="I62" s="9" t="n">
+        <f aca="false">IFERROR(H62-A62,"")</f>
         <v>-4</v>
       </c>
     </row>
@@ -4256,12 +4966,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A63,מקור!$L$2:$L$309,0)),"")</f>
         <v>5642.9</v>
       </c>
-      <c r="E63" s="5" t="n">
+      <c r="E63" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A63,מקור!$L$2:$L$309,0)),"")</f>
+        <v>11540.6</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <f aca="false">IFERROR(E63/12*6,"")</f>
+        <v>5770.3</v>
+      </c>
+      <c r="G63" s="7" t="n">
+        <f aca="false">IFERROR(D63/F63-1,"")</f>
+        <v>-0.0220785747708092</v>
+      </c>
+      <c r="H63" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A63,מקור!$L$2:$L$309,0)),"")</f>
         <v>56</v>
       </c>
-      <c r="F63" s="9" t="n">
-        <f aca="false">IFERROR(E63-A63,"")</f>
+      <c r="I63" s="9" t="n">
+        <f aca="false">IFERROR(H63-A63,"")</f>
         <v>-3</v>
       </c>
     </row>
@@ -4281,12 +5003,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A64,מקור!$L$2:$L$309,0)),"")</f>
         <v>4316.1</v>
       </c>
-      <c r="E64" s="5" t="n">
+      <c r="E64" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A64,מקור!$L$2:$L$309,0)),"")</f>
+        <v>11428.1</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <f aca="false">IFERROR(E64/12*6,"")</f>
+        <v>5714.05</v>
+      </c>
+      <c r="G64" s="7" t="n">
+        <f aca="false">IFERROR(D64/F64-1,"")</f>
+        <v>-0.244651341867852</v>
+      </c>
+      <c r="H64" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A64,מקור!$L$2:$L$309,0)),"")</f>
         <v>61</v>
       </c>
-      <c r="F64" s="9" t="n">
-        <f aca="false">IFERROR(E64-A64,"")</f>
+      <c r="I64" s="9" t="n">
+        <f aca="false">IFERROR(H64-A64,"")</f>
         <v>1</v>
       </c>
     </row>
@@ -4306,12 +5040,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A65,מקור!$L$2:$L$309,0)),"")</f>
         <v>4994.4</v>
       </c>
-      <c r="E65" s="5" t="n">
+      <c r="E65" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A65,מקור!$L$2:$L$309,0)),"")</f>
+        <v>10880.1</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <f aca="false">IFERROR(E65/12*6,"")</f>
+        <v>5440.05</v>
+      </c>
+      <c r="G65" s="7" t="n">
+        <f aca="false">IFERROR(D65/F65-1,"")</f>
+        <v>-0.0819202029393114</v>
+      </c>
+      <c r="H65" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A65,מקור!$L$2:$L$309,0)),"")</f>
         <v>59</v>
       </c>
-      <c r="F65" s="9" t="n">
-        <f aca="false">IFERROR(E65-A65,"")</f>
+      <c r="I65" s="9" t="n">
+        <f aca="false">IFERROR(H65-A65,"")</f>
         <v>-2</v>
       </c>
     </row>
@@ -4331,12 +5077,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A66,מקור!$L$2:$L$309,0)),"")</f>
         <v>2856.9</v>
       </c>
-      <c r="E66" s="5" t="n">
+      <c r="E66" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A66,מקור!$L$2:$L$309,0)),"")</f>
+        <v>16006.4</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <f aca="false">IFERROR(E66/12*6,"")</f>
+        <v>8003.2</v>
+      </c>
+      <c r="G66" s="7" t="n">
+        <f aca="false">IFERROR(D66/F66-1,"")</f>
+        <v>-0.643030287884846</v>
+      </c>
+      <c r="H66" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A66,מקור!$L$2:$L$309,0)),"")</f>
         <v>65</v>
       </c>
-      <c r="F66" s="9" t="n">
-        <f aca="false">IFERROR(E66-A66,"")</f>
+      <c r="I66" s="9" t="n">
+        <f aca="false">IFERROR(H66-A66,"")</f>
         <v>3</v>
       </c>
     </row>
@@ -4356,12 +5114,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A67,מקור!$L$2:$L$309,0)),"")</f>
         <v>3276.5</v>
       </c>
-      <c r="E67" s="5" t="n">
+      <c r="E67" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A67,מקור!$L$2:$L$309,0)),"")</f>
+        <v>2655</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <f aca="false">IFERROR(E67/12*6,"")</f>
+        <v>1327.5</v>
+      </c>
+      <c r="G67" s="7" t="n">
+        <f aca="false">IFERROR(D67/F67-1,"")</f>
+        <v>1.46817325800377</v>
+      </c>
+      <c r="H67" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A67,מקור!$L$2:$L$309,0)),"")</f>
         <v>63</v>
       </c>
-      <c r="F67" s="9" t="n">
-        <f aca="false">IFERROR(E67-A67,"")</f>
+      <c r="I67" s="9" t="n">
+        <f aca="false">IFERROR(H67-A67,"")</f>
         <v>0</v>
       </c>
     </row>
@@ -4381,12 +5151,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A68,מקור!$L$2:$L$309,0)),"")</f>
         <v>2637</v>
       </c>
-      <c r="E68" s="5" t="n">
+      <c r="E68" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A68,מקור!$L$2:$L$309,0)),"")</f>
+        <v>7486.3</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <f aca="false">IFERROR(E68/12*6,"")</f>
+        <v>3743.15</v>
+      </c>
+      <c r="G68" s="7" t="n">
+        <f aca="false">IFERROR(D68/F68-1,"")</f>
+        <v>-0.295513137330858</v>
+      </c>
+      <c r="H68" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A68,מקור!$L$2:$L$309,0)),"")</f>
         <v>66</v>
       </c>
-      <c r="F68" s="9" t="n">
-        <f aca="false">IFERROR(E68-A68,"")</f>
+      <c r="I68" s="9" t="n">
+        <f aca="false">IFERROR(H68-A68,"")</f>
         <v>2</v>
       </c>
     </row>
@@ -4406,12 +5188,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A69,מקור!$L$2:$L$309,0)),"")</f>
         <v>3663</v>
       </c>
-      <c r="E69" s="5" t="n">
+      <c r="E69" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A69,מקור!$L$2:$L$309,0)),"")</f>
+        <v>9185.3</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <f aca="false">IFERROR(E69/12*6,"")</f>
+        <v>4592.65</v>
+      </c>
+      <c r="G69" s="7" t="n">
+        <f aca="false">IFERROR(D69/F69-1,"")</f>
+        <v>-0.20242126005683</v>
+      </c>
+      <c r="H69" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A69,מקור!$L$2:$L$309,0)),"")</f>
         <v>62</v>
       </c>
-      <c r="F69" s="9" t="n">
-        <f aca="false">IFERROR(E69-A69,"")</f>
+      <c r="I69" s="9" t="n">
+        <f aca="false">IFERROR(H69-A69,"")</f>
         <v>-3</v>
       </c>
     </row>
@@ -4431,12 +5225,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A70,מקור!$L$2:$L$309,0)),"")</f>
         <v>1835.1</v>
       </c>
-      <c r="E70" s="5" t="n">
+      <c r="E70" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A70,מקור!$L$2:$L$309,0)),"")</f>
+        <v>2534.6</v>
+      </c>
+      <c r="F70" s="6" t="n">
+        <f aca="false">IFERROR(E70/12*6,"")</f>
+        <v>1267.3</v>
+      </c>
+      <c r="G70" s="7" t="n">
+        <f aca="false">IFERROR(D70/F70-1,"")</f>
+        <v>0.448039138325574</v>
+      </c>
+      <c r="H70" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A70,מקור!$L$2:$L$309,0)),"")</f>
         <v>68</v>
       </c>
-      <c r="F70" s="9" t="n">
-        <f aca="false">IFERROR(E70-A70,"")</f>
+      <c r="I70" s="9" t="n">
+        <f aca="false">IFERROR(H70-A70,"")</f>
         <v>2</v>
       </c>
     </row>
@@ -4456,12 +5262,24 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A71,מקור!$L$2:$L$309,0)),"")</f>
         <v>2907.8</v>
       </c>
-      <c r="E71" s="5" t="n">
+      <c r="E71" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A71,מקור!$L$2:$L$309,0)),"")</f>
+        <v>6815</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <f aca="false">IFERROR(E71/12*6,"")</f>
+        <v>3407.5</v>
+      </c>
+      <c r="G71" s="7" t="n">
+        <f aca="false">IFERROR(D71/F71-1,"")</f>
+        <v>-0.146647101980924</v>
+      </c>
+      <c r="H71" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A71,מקור!$L$2:$L$309,0)),"")</f>
         <v>64</v>
       </c>
-      <c r="F71" s="9" t="n">
-        <f aca="false">IFERROR(E71-A71,"")</f>
+      <c r="I71" s="9" t="n">
+        <f aca="false">IFERROR(H71-A71,"")</f>
         <v>-3</v>
       </c>
     </row>
@@ -4481,16 +5299,28 @@
         <f aca="false">IFERROR(INDEX(מקור!$I$2:$I$309,MATCH("דודו|"&amp;A72,מקור!$L$2:$L$309,0)),"")</f>
         <v>2594.7</v>
       </c>
-      <c r="E72" s="5" t="n">
+      <c r="E72" s="6" t="n">
+        <f aca="false">IFERROR(INDEX(מקור!$J$2:$J$309,MATCH("דודו|"&amp;A72,מקור!$L$2:$L$309,0)),"")</f>
+        <v>0</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <f aca="false">IFERROR(E72/12*6,"")</f>
+        <v>0</v>
+      </c>
+      <c r="G72" s="7" t="str">
+        <f aca="false">IFERROR(D72/F72-1,"")</f>
+        <v/>
+      </c>
+      <c r="H72" s="5" t="n">
         <f aca="false">IFERROR(INDEX(מקור!$M$2:$M$309,MATCH("דודו|"&amp;A72,מקור!$L$2:$L$309,0)),"")</f>
         <v>67</v>
       </c>
-      <c r="F72" s="9" t="n">
-        <f aca="false">IFERROR(E72-A72,"")</f>
+      <c r="I72" s="9" t="n">
+        <f aca="false">IFERROR(H72-A72,"")</f>
         <v>-1</v>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="s">
         <v>18</v>
       </c>
@@ -4499,15 +5329,18 @@
       <c r="D74" s="8"/>
       <c r="E74" s="8"/>
       <c r="F74" s="8"/>
+      <c r="G74" s="8"/>
+      <c r="H74" s="8"/>
+      <c r="I74" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A74:F74"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A74:I74"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:F72">
+  <conditionalFormatting sqref="A5:I72">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
-      <formula>AND(ISNUMBER($F5),$F5&gt;=10)</formula>
+      <formula>AND(ISNUMBER($I5),$I5&gt;=10)</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>